<commit_message>
Update all pending changes
</commit_message>
<xml_diff>
--- a/SAB Campus Dashboard.xlsx
+++ b/SAB Campus Dashboard.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\bom tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://casrilanka-my.sharepoint.com/personal/salinda_wickramasinghe_sab_casrilanka_com/Documents/Salinda Wickramasinghe/Projects/Project/bom tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B2AD02-BA9F-4893-AEB9-E9B306EDED7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{CC0CEE26-EAC3-4A34-BD9E-2ADA82BCA8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA72E843-1E35-4AE3-8355-7475E52137D4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lecture_Breakdown" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,8 @@
     <sheet name="Lecture_Endings" sheetId="8" r:id="rId8"/>
     <sheet name="Internship" sheetId="9" r:id="rId9"/>
     <sheet name="Counselling sessions " sheetId="10" r:id="rId10"/>
+    <sheet name="Meetings" sheetId="11" r:id="rId11"/>
+    <sheet name="New Recruitment" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,8 +46,90 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="7">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="7">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="139">
   <si>
     <t>Degree</t>
   </si>
@@ -71,265 +155,334 @@
     <t>Exam_Cycle</t>
   </si>
   <si>
+    <t>No of Exam Papers</t>
+  </si>
+  <si>
+    <t>Results Released</t>
+  </si>
+  <si>
+    <t>Complete percentage</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t xml:space="preserve">February </t>
+  </si>
+  <si>
+    <t>No. of Exams</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venue </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reource Person </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualifications </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guest Lecture Topic </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Subject </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch </t>
+  </si>
+  <si>
+    <t>7th February 2026</t>
+  </si>
+  <si>
+    <t>3.30pm - 6.30 pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Roshan Jayantha </t>
+  </si>
+  <si>
+    <t>Fellow chartered accounted (FCA), Phd,MBA</t>
+  </si>
+  <si>
+    <t>From Research Problem to Data Collection: A Practical Workshop for Research Students</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dissertation (4Y. 2 Sem) </t>
+  </si>
+  <si>
+    <t>15 D (WE), 16A (MOHE), 16B (WE)(WD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20th February 2026 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.00 am - 12.00 noon </t>
+  </si>
+  <si>
+    <t>SAB</t>
+  </si>
+  <si>
+    <t>Mr. Nishantha Bandara Illangasinghe</t>
+  </si>
+  <si>
+    <t>Head - Strategic Development Unit, Hayleys Agriculture Holdings Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sustainability Accounting in Practice: The Accountant’s Role </t>
+  </si>
+  <si>
+    <t>Advanced Management Accounting(2 Y 2 sem)</t>
+  </si>
+  <si>
+    <t>18B WD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18th March 2026 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.30 am - 12.30 noon </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAB </t>
+  </si>
+  <si>
+    <t>Eng.Janaka Rathnakumara</t>
+  </si>
+  <si>
+    <t>COO - Wijeya Newspapers Ltd. (CE,CEP,MSc,BSc)</t>
+  </si>
+  <si>
+    <t>Bridging Sustainability Actions and Financial Reporting</t>
+  </si>
+  <si>
+    <t>Financial Reporting (2 Y 1 sem)</t>
+  </si>
+  <si>
+    <t>19A (WD)</t>
+  </si>
+  <si>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>Thai Pongal</t>
+  </si>
+  <si>
+    <t>8th Feb</t>
+  </si>
+  <si>
+    <t>Blood Doation Campaign</t>
+  </si>
+  <si>
+    <t>13th Feb</t>
+  </si>
+  <si>
+    <t>10th IFSL Intake Students Registration</t>
+  </si>
+  <si>
+    <t>11th March</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iftar Celebration </t>
+  </si>
+  <si>
+    <t>Inauguration Ceremony Intake 20A &amp; 4A</t>
+  </si>
+  <si>
+    <t>21st March</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achivements </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sports - Runners-up CPA Cricket Tournament </t>
+  </si>
+  <si>
+    <t>Academics - CFA Institute Research Challenge</t>
+  </si>
+  <si>
+    <t>Degree Programme</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>Cumulative</t>
+  </si>
+  <si>
+    <t> Oct</t>
+  </si>
+  <si>
+    <t>Cum. Total</t>
+  </si>
+  <si>
+    <t>(Aug)</t>
+  </si>
+  <si>
+    <t>Applied Accounting</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>MoHE</t>
+  </si>
+  <si>
+    <t>(Applied Accounting)</t>
+  </si>
+  <si>
+    <t>Exemptions</t>
+  </si>
+  <si>
+    <t>Business Analytics</t>
+  </si>
+  <si>
+    <t>MoHE (Business Analytics)</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Applications received</t>
+  </si>
+  <si>
+    <t>MoHE Selected applicants</t>
+  </si>
+  <si>
+    <t>Registered applicants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Accounting </t>
+  </si>
+  <si>
+    <t>221*</t>
+  </si>
+  <si>
+    <t>82*</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month </t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
     <t>Jan</t>
   </si>
   <si>
     <t>Feb</t>
   </si>
   <si>
-    <t>March</t>
-  </si>
-  <si>
-    <t>July</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Cumulative</t>
-  </si>
-  <si>
-    <t>Target</t>
-  </si>
-  <si>
-    <t>Cum. Total</t>
-  </si>
-  <si>
-    <t>Applied Accounting</t>
-  </si>
-  <si>
-    <t>Budget</t>
-  </si>
-  <si>
-    <t>Actual</t>
-  </si>
-  <si>
-    <t>MoHE</t>
-  </si>
-  <si>
-    <t>(Applied Accounting)</t>
-  </si>
-  <si>
-    <t>Exemptions</t>
-  </si>
-  <si>
-    <t>MoHE (Business Analytics)</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>Y1 S2</t>
+    <t xml:space="preserve">Jan </t>
+  </si>
+  <si>
+    <t>Batch</t>
+  </si>
+  <si>
+    <t>Y:S</t>
+  </si>
+  <si>
+    <t>New Semester commencement</t>
+  </si>
+  <si>
+    <t>17C WD/WE</t>
+  </si>
+  <si>
+    <t>Y3 S2</t>
+  </si>
+  <si>
+    <t>19A WE /MOHE WE</t>
+  </si>
+  <si>
+    <t>Y2 S1</t>
+  </si>
+  <si>
+    <t>3AWE /MOHE WE (BMBA)</t>
+  </si>
+  <si>
+    <t>20A MOHE WD</t>
+  </si>
+  <si>
+    <t>Y1 S1</t>
+  </si>
+  <si>
+    <t>20A WD</t>
+  </si>
+  <si>
+    <t>4A WD/MOHE WD (BMBA)</t>
+  </si>
+  <si>
+    <t>18C WD</t>
   </si>
   <si>
     <t>Y2 S2</t>
   </si>
   <si>
-    <t>18B WD</t>
-  </si>
-  <si>
-    <t>Y2 S1</t>
-  </si>
-  <si>
-    <t>Results Released</t>
-  </si>
-  <si>
-    <t>No of Exam Papers</t>
-  </si>
-  <si>
-    <t>September</t>
-  </si>
-  <si>
-    <t>October</t>
-  </si>
-  <si>
-    <t>November</t>
-  </si>
-  <si>
-    <t>January</t>
-  </si>
-  <si>
-    <t>No.</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venue </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reource Person </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qualifications </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guest Lecture Topic </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Subject </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Batch </t>
-  </si>
-  <si>
-    <t>7th February 2026</t>
-  </si>
-  <si>
-    <t>3.30pm - 6.30 pm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr. Roshan Jayantha </t>
-  </si>
-  <si>
-    <t>From Research Problem to Data Collection: A Practical Workshop for Research Students</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dissertation (4Y. 2 Sem) </t>
-  </si>
-  <si>
-    <t>15 D (WE), 16A (MOHE), 16B (WE)(WD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20th February 2026 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.00 am - 12.00 noon </t>
-  </si>
-  <si>
-    <t>SAB</t>
-  </si>
-  <si>
-    <t>Mr. Nishantha Bandara Illangasinghe</t>
-  </si>
-  <si>
-    <t>Head - Strategic Development Unit, Hayleys Agriculture Holdings Ltd.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sustainability Accounting in Practice: The Accountant’s Role </t>
-  </si>
-  <si>
-    <t>Advanced Management Accounting(2 Y 2 sem)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18th March 2026 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.30 am - 12.30 noon </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAB </t>
-  </si>
-  <si>
-    <t>Bridging Sustainability Actions and Financial Reporting</t>
-  </si>
-  <si>
-    <t>Financial Reporting (2 Y 1 sem)</t>
-  </si>
-  <si>
-    <t>19A (WD)</t>
-  </si>
-  <si>
-    <t>COO - Wijeya Newspapers Ltd. (CE,CEP,MSc,BSc)</t>
-  </si>
-  <si>
-    <t>Eng.Janaka Rathnakumara</t>
-  </si>
-  <si>
-    <t>Fellow chartered accounted (FCA), Phd,MBA</t>
-  </si>
-  <si>
-    <t>Event</t>
-  </si>
-  <si>
-    <t>Thai Pongal</t>
-  </si>
-  <si>
-    <t>8th Feb</t>
-  </si>
-  <si>
-    <t>13th Feb</t>
-  </si>
-  <si>
-    <t>Blood Doation Campaign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iftar Celebration </t>
-  </si>
-  <si>
-    <t>14th March</t>
-  </si>
-  <si>
-    <t>Degree Programme</t>
-  </si>
-  <si>
-    <t>(Aug)</t>
-  </si>
-  <si>
-    <t> Oct</t>
-  </si>
-  <si>
-    <t>Business Analytics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Month </t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan </t>
-  </si>
-  <si>
-    <t>Batch</t>
-  </si>
-  <si>
-    <t>Y:S</t>
-  </si>
-  <si>
-    <t>New Semester commencement</t>
-  </si>
-  <si>
-    <t>19B Ex</t>
-  </si>
-  <si>
-    <t>17B MOHE WD/WE</t>
-  </si>
-  <si>
-    <t>Y3 S2</t>
-  </si>
-  <si>
-    <t>19B MOHE WE</t>
-  </si>
-  <si>
-    <t>19B WE </t>
-  </si>
-  <si>
-    <t>3BWE /MOHE WE (BMBA)</t>
-  </si>
-  <si>
-    <t>18B WE</t>
-  </si>
-  <si>
-    <t>2B WD/WE (BMBA)</t>
-  </si>
-  <si>
-    <t>19A WD/MOHE WD</t>
-  </si>
-  <si>
-    <t>3A WD/MOHE WD (BMBA)</t>
-  </si>
-  <si>
-    <t>18A WE/18C EX - CA,MAAT</t>
-  </si>
-  <si>
-    <t>2A WE (BMBA)</t>
-  </si>
-  <si>
-    <t>End Semester  </t>
+    <t>20A MOHE WE</t>
+  </si>
+  <si>
+    <t>End Semester </t>
+  </si>
+  <si>
+    <t>18C WE</t>
+  </si>
+  <si>
+    <t>2C WE  (BMBA)</t>
+  </si>
+  <si>
+    <t>16A MOHE WE/WD,16C /D WD WE ,17BEX ,18A EX</t>
+  </si>
+  <si>
+    <t>Y4 S1</t>
+  </si>
+  <si>
+    <t>19C WD</t>
+  </si>
+  <si>
+    <t>19C WE</t>
+  </si>
+  <si>
+    <t>3C WE (BMBA)</t>
+  </si>
+  <si>
+    <t>15D WE and 16A MOHE WD, 16B WD/WE</t>
+  </si>
+  <si>
+    <t>Y4 S2</t>
   </si>
   <si>
     <t>Audit</t>
@@ -344,22 +497,55 @@
     <t>Non Audit</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t xml:space="preserve">CA Registered </t>
   </si>
   <si>
     <t>CA Not Registred</t>
   </si>
   <si>
+    <t>EY</t>
+  </si>
+  <si>
+    <t>Deloitte</t>
+  </si>
+  <si>
+    <t>KPMG</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
     <t>Counselling sessions </t>
   </si>
   <si>
-    <t>Month</t>
-  </si>
-  <si>
-    <t>Complete percentage</t>
+    <t>Meeting</t>
+  </si>
+  <si>
+    <t>No. Meeting</t>
+  </si>
+  <si>
+    <t>Board of Management</t>
+  </si>
+  <si>
+    <t>Board of Studies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audit Committee Meeting </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name </t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasitha Karunarathna </t>
+  </si>
+  <si>
+    <t>Deputy Registrar – Examinations</t>
+  </si>
+  <si>
+    <t>15th March</t>
   </si>
 </sst>
 </file>
@@ -368,9 +554,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -452,8 +638,34 @@
       <color rgb="FF000000"/>
       <name val="Inherit"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -484,8 +696,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="24">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -750,11 +968,72 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
@@ -762,27 +1041,14 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -792,7 +1058,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -856,27 +1122,77 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="12" fillId="6" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -910,28 +1226,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -939,19 +1234,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -970,6 +1252,100 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="7">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1282,7 +1658,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="2">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1293,7 +1669,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="2">
-        <v>95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1304,7 +1680,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="2">
-        <v>113</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1315,7 +1691,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="2">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1325,7 +1701,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F86E63A4-FAA2-4D5C-9A3F-1AF6A2363593}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
@@ -1333,16 +1709,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="30" t="s">
-        <v>102</v>
+      <c r="A1" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="B2" s="2">
         <v>9</v>
@@ -1350,10 +1726,94 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>91</v>
       </c>
       <c r="B3" s="2">
         <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="2">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00AA665D-2D81-43C0-8BFF-AA187832AC2C}">
+  <dimension ref="B2:C5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3">
+      <c r="B2" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A217B18-E3F7-4280-B7D4-04E1202D6CDC}">
+  <dimension ref="B4:C5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:3">
+      <c r="B4" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1363,10 +1823,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
     <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
@@ -1377,18 +1837,18 @@
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="53" t="s">
-        <v>104</v>
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2">
         <v>42</v>
@@ -1396,14 +1856,14 @@
       <c r="C2" s="2">
         <v>42</v>
       </c>
-      <c r="D2" s="54">
+      <c r="D2" s="27">
         <f>C2/B2*100</f>
         <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2">
         <v>30</v>
@@ -1411,14 +1871,14 @@
       <c r="C3" s="2">
         <v>30</v>
       </c>
-      <c r="D3" s="54">
-        <f t="shared" ref="D3:D5" si="0">C3/B3*100</f>
+      <c r="D3" s="27">
+        <f t="shared" ref="D3:D6" si="0">C3/B3*100</f>
         <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2">
         <v>17</v>
@@ -1426,24 +1886,87 @@
       <c r="C4" s="2">
         <v>17</v>
       </c>
-      <c r="D4" s="54">
+      <c r="D4" s="27">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2">
         <v>50</v>
       </c>
       <c r="C5" s="2">
-        <v>9</v>
-      </c>
-      <c r="D5" s="54">
+        <v>40</v>
+      </c>
+      <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2">
+        <v>34</v>
+      </c>
+      <c r="C6" s="2">
+        <v>5</v>
+      </c>
+      <c r="D6" s="28">
+        <f t="shared" si="0"/>
+        <v>14.705882352941178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="38">
+        <v>45658</v>
+      </c>
+      <c r="B10" s="39">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="38">
+        <v>45689</v>
+      </c>
+      <c r="B11" s="39">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="38">
+        <v>45717</v>
+      </c>
+      <c r="B12" s="39">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="38">
+        <v>45748</v>
+      </c>
+      <c r="B13" s="39">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="38">
+        <v>45778</v>
+      </c>
+      <c r="B14" s="39">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1454,44 +1977,44 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.28515625" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="6" max="10" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30">
+    <row r="1" spans="1:9">
       <c r="A1" s="3" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60">
@@ -1499,118 +2022,173 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="90">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="60">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="60">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="45">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="B7" s="5" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <v>18</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="61.15" customHeight="1">
       <c r="B8" s="5" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>53</v>
+      </c>
+      <c r="D8" s="2" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="61.15" customHeight="1">
       <c r="B9" s="5" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+        <v>55</v>
+      </c>
+      <c r="D9" s="2" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="61.9" customHeight="1">
       <c r="B10" s="5" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>71</v>
+        <v>57</v>
+      </c>
+      <c r="D10" s="2" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="61.15" customHeight="1">
+      <c r="B11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" s="2" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="62.45" customHeight="1">
+      <c r="B12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="2" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="B15" s="35" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="85.15" customHeight="1">
+      <c r="B16" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="2" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" ht="63.6" customHeight="1">
+      <c r="B17" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="2" t="e" vm="7">
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -1633,45 +2211,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="46" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="48" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="48" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="42" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A2" s="47"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="49"/>
+      <c r="G2" s="43"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A3" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="49" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="49" t="s">
-        <v>74</v>
-      </c>
-      <c r="G1" s="43" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>73</v>
-      </c>
-      <c r="F2" s="50"/>
-      <c r="G2" s="44"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1">
-      <c r="A3" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>17</v>
       </c>
       <c r="C3" s="9">
         <v>100</v>
@@ -1690,12 +2268,12 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="24.6" customHeight="1" thickBot="1">
-      <c r="A4" s="46"/>
+      <c r="A4" s="45"/>
       <c r="B4" s="8" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="C4" s="10">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10">
@@ -1708,10 +2286,10 @@
     </row>
     <row r="5" spans="1:7" ht="12.6" customHeight="1" thickBot="1">
       <c r="A5" s="13" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9">
@@ -1727,10 +2305,10 @@
     </row>
     <row r="6" spans="1:7" ht="24.6" customHeight="1" thickBot="1">
       <c r="A6" s="16" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
@@ -1739,11 +2317,11 @@
       <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" ht="12.6" customHeight="1" thickBot="1">
-      <c r="A7" s="45" t="s">
-        <v>21</v>
+      <c r="A7" s="44" t="s">
+        <v>77</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9">
@@ -1758,22 +2336,24 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="12.6" customHeight="1" thickBot="1">
-      <c r="A8" s="46"/>
+      <c r="A8" s="45"/>
       <c r="B8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="10"/>
+        <v>74</v>
+      </c>
+      <c r="C8" s="10">
+        <v>21</v>
+      </c>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="11"/>
       <c r="G8" s="15"/>
     </row>
     <row r="9" spans="1:7" ht="12.6" customHeight="1" thickBot="1">
-      <c r="A9" s="45" t="s">
-        <v>75</v>
+      <c r="A9" s="44" t="s">
+        <v>78</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="C9" s="9">
         <v>50</v>
@@ -1790,12 +2370,12 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="13.9" customHeight="1" thickBot="1">
-      <c r="A10" s="46"/>
+      <c r="A10" s="45"/>
       <c r="B10" s="8" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="C10" s="10">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10">
@@ -1807,11 +2387,11 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="12.6" customHeight="1" thickBot="1">
-      <c r="A11" s="45" t="s">
-        <v>22</v>
+      <c r="A11" s="44" t="s">
+        <v>79</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9">
@@ -1826,9 +2406,9 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.9" customHeight="1" thickBot="1">
-      <c r="A12" s="46"/>
+      <c r="A12" s="45"/>
       <c r="B12" s="8" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -1837,11 +2417,11 @@
       <c r="G12" s="15"/>
     </row>
     <row r="13" spans="1:7" ht="12.6" customHeight="1" thickBot="1">
-      <c r="A13" s="36" t="s">
-        <v>23</v>
+      <c r="A13" s="54" t="s">
+        <v>80</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="C13" s="9">
         <v>150</v>
@@ -1860,40 +2440,96 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="24.6" customHeight="1">
-      <c r="A14" s="37"/>
-      <c r="B14" s="39" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="41">
+      <c r="A14" s="55"/>
+      <c r="B14" s="57" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="59">
+        <f>C10+C8+C4</f>
+        <v>202</v>
+      </c>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59">
         <v>116</v>
       </c>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41">
+      <c r="F14" s="50"/>
+      <c r="G14" s="52">
         <v>116</v>
       </c>
-      <c r="F14" s="32"/>
-      <c r="G14" s="34">
-        <v>116</v>
-      </c>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="38"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="35"/>
+      <c r="A15" s="56"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="60"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="53"/>
     </row>
     <row r="16" spans="1:7" ht="12.6" customHeight="1"/>
-    <row r="17" ht="12.6" customHeight="1"/>
-    <row r="18" ht="12.6" customHeight="1"/>
-    <row r="19" ht="12.6" customHeight="1"/>
-    <row r="20" ht="12.6" customHeight="1"/>
-    <row r="21" ht="12.6" customHeight="1"/>
-    <row r="22" ht="12.6" customHeight="1"/>
+    <row r="17" spans="1:4" ht="12.6" customHeight="1" thickBot="1"/>
+    <row r="18" spans="1:4" ht="36.75" thickBot="1">
+      <c r="A18" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="23.45" customHeight="1" thickBot="1">
+      <c r="A19" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="32">
+        <v>294</v>
+      </c>
+      <c r="C19" s="32">
+        <v>279</v>
+      </c>
+      <c r="D19" s="32" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="17.45" customHeight="1">
+      <c r="A20" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="34">
+        <v>100</v>
+      </c>
+      <c r="C20" s="34">
+        <v>100</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="12.6" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="12.6" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A7:A8"/>
@@ -1904,13 +2540,6 @@
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="F1:F2"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1918,20 +2547,20 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>77</v>
+      <c r="A1" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="B2" s="2">
         <v>15</v>
@@ -1939,10 +2568,18 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>91</v>
       </c>
       <c r="B3" s="2">
         <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="2">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1952,23 +2589,31 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="B2" s="2">
         <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1978,7 +2623,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -1988,131 +2633,119 @@
     <col min="5" max="5" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75">
-      <c r="A2" s="55" t="s">
-        <v>81</v>
-      </c>
-      <c r="B2" s="25">
-        <v>46060</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="14.45" customHeight="1">
-      <c r="A3" s="56"/>
-      <c r="B3" s="25">
-        <v>46060</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A4" s="56"/>
-      <c r="B4" s="25">
-        <v>46060</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>24</v>
+    <row r="1" spans="1:4" ht="14.45" customHeight="1">
+      <c r="A1" s="40"/>
+      <c r="B1" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" s="41" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="14.45" customHeight="1">
+      <c r="A2" s="61" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="17">
+        <v>46088</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A3" s="61"/>
+      <c r="B3" s="20">
+        <v>46095</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75">
+      <c r="A4" s="61"/>
+      <c r="B4" s="20">
+        <v>46095</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75">
-      <c r="A5" s="56"/>
-      <c r="B5" s="25">
-        <v>46060</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="27" t="s">
-        <v>24</v>
+      <c r="A5" s="61"/>
+      <c r="B5" s="20">
+        <v>46104</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75">
-      <c r="A6" s="56"/>
-      <c r="B6" s="25">
-        <v>46060</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>24</v>
+      <c r="A6" s="61"/>
+      <c r="B6" s="20">
+        <v>46104</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75">
-      <c r="A7" s="56"/>
-      <c r="B7" s="25">
-        <v>46067</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="27" t="s">
-        <v>25</v>
+      <c r="A7" s="61"/>
+      <c r="B7" s="20">
+        <v>46104</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75">
-      <c r="A8" s="56"/>
-      <c r="B8" s="25">
-        <v>46067</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="D8" s="27" t="s">
-        <v>25</v>
+      <c r="A8" s="61"/>
+      <c r="B8" s="20">
+        <v>46106</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75">
-      <c r="A9" s="56"/>
-      <c r="B9" s="25">
-        <v>46077</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75">
-      <c r="A10" s="57"/>
-      <c r="B10" s="25">
-        <v>46078</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>27</v>
+      <c r="A9" s="61"/>
+      <c r="B9" s="20">
+        <v>46109</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="A2:A9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2120,7 +2753,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="B2:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -2129,46 +2762,106 @@
     <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75">
-      <c r="B1" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75">
-      <c r="A2" s="51" t="s">
+    <row r="2" spans="2:5" ht="15.75">
+      <c r="C2" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="17">
-        <v>46061</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75">
-      <c r="A3" s="52"/>
-      <c r="B3" s="20">
-        <v>46061</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>25</v>
+    </row>
+    <row r="3" spans="2:5" ht="15.75">
+      <c r="B3" s="62" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="17">
+        <v>46082</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="15.75">
+      <c r="B4" s="63"/>
+      <c r="C4" s="20">
+        <v>46082</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="15.75">
+      <c r="B5" s="63"/>
+      <c r="C5" s="20">
+        <v>46082</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="15.75">
+      <c r="B6" s="63"/>
+      <c r="C6" s="20">
+        <v>46086</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="15.75">
+      <c r="B7" s="63"/>
+      <c r="C7" s="20">
+        <v>46096</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="15.75">
+      <c r="B8" s="63"/>
+      <c r="C8" s="20">
+        <v>46096</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="15.75">
+      <c r="B9" s="63"/>
+      <c r="C9" s="20">
+        <v>46088</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B3:B9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2176,7 +2869,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01DE9DF-231D-4D5D-B012-EDD3B658E061}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
@@ -2185,7 +2878,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="B1" s="2">
         <v>268</v>
@@ -2193,7 +2886,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="B2" s="2">
         <v>85</v>
@@ -2201,7 +2894,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="B3" s="2">
         <v>236</v>
@@ -2209,7 +2902,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="B4" s="2">
         <v>249</v>
@@ -2217,7 +2910,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="B5" s="2">
         <v>517</v>
@@ -2225,46 +2918,70 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="B7" s="2">
         <v>268</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="23">
         <v>0.52</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="B8" s="2">
         <v>249</v>
       </c>
-      <c r="C8" s="28">
+      <c r="C8" s="23">
         <v>0.48</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="B10" s="2">
         <v>423</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="24">
         <v>0.82</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="B11" s="2">
         <v>94</v>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="24">
         <v>0.18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="2">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>